<commit_message>
Senior: quita la T21 y deja la T22 con sus números de la jornada 1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0194DjF3wyQR2qJcGdkm9Jw4
</commit_message>
<xml_diff>
--- a/senior-numeros.xlsx
+++ b/senior-numeros.xlsx
@@ -11,10 +11,10 @@
     <sheet name="Léeme" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Tabla" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Resultados" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Team Trampa" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="White Lions" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Fantasía" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Colegio Javier" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Deejays" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="La Pandilla" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Cerveceros" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Fantasía" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="122">
   <si>
     <t xml:space="preserve">Números del Meracho Senior · La Mella League</t>
   </si>
@@ -34,13 +34,13 @@
     <t xml:space="preserve">Liga</t>
   </si>
   <si>
-    <t xml:space="preserve">Meracho Senior · Temporada 21 · miércoles en el Complejo Deportivo del MEF, Albrook</t>
+    <t xml:space="preserve">Meracho Senior · Temporada 22 · miércoles en el Complejo Deportivo del MEF, Albrook</t>
   </si>
   <si>
     <t xml:space="preserve">Corte</t>
   </si>
   <si>
-    <t xml:space="preserve">Después de la jornada 3 (miércoles 30 de septiembre de 2026) · fin de la fase de grupos</t>
+    <t xml:space="preserve">Después de la jornada 1 (miércoles 21 de octubre de 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Desarrollo</t>
@@ -58,10 +58,10 @@
     <t xml:space="preserve">Juegos jugados</t>
   </si>
   <si>
-    <t xml:space="preserve">AP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apariciones al plato</t>
+    <t xml:space="preserve">VB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Veces al bate</t>
   </si>
   <si>
     <t xml:space="preserve">H</t>
@@ -163,19 +163,19 @@
     <t xml:space="preserve">1</t>
   </si>
   <si>
-    <t xml:space="preserve">Team Trampa</t>
+    <t xml:space="preserve">Deejays</t>
   </si>
   <si>
     <t xml:space="preserve">2</t>
   </si>
   <si>
-    <t xml:space="preserve">White Lions</t>
+    <t xml:space="preserve">La Pandilla</t>
   </si>
   <si>
     <t xml:space="preserve">3</t>
   </si>
   <si>
-    <t xml:space="preserve">Colegio Javier</t>
+    <t xml:space="preserve">Cerveceros</t>
   </si>
   <si>
     <t xml:space="preserve">4</t>
@@ -184,7 +184,7 @@
     <t xml:space="preserve">Fantasía</t>
   </si>
   <si>
-    <t xml:space="preserve">Fin de la fase de grupos (jornada 3): sin empates en la tabla, no hace falta desempate. Semifinales del miércoles 7 de octubre: 7:30 Fantasía (4.º) en casa de Team Trampa (1.º) · 9:00 Colegio Javier (3.º) en casa de White Lions (2.º).</t>
+    <t xml:space="preserve">Después de la jornada 1: Deejays y La Pandilla 1-0, Cerveceros y Fantasía 0-1. Los empatados no se han enfrentado: los separa la diferencia global de carreras. Jornada 2, miércoles 28 de octubre: 7:30 Fantasía vs Cerveceros · 9:00 Deejays vs La Pandilla.</t>
   </si>
   <si>
     <t xml:space="preserve">Resultados</t>
@@ -214,7 +214,7 @@
     <t xml:space="preserve">Entradas</t>
   </si>
   <si>
-    <t xml:space="preserve">mié 16 sep</t>
+    <t xml:space="preserve">mié 21 oct</t>
   </si>
   <si>
     <t xml:space="preserve">7:30 pm</t>
@@ -223,229 +223,175 @@
     <t xml:space="preserve">9:00 pm</t>
   </si>
   <si>
-    <t xml:space="preserve">mié 23 sep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mié 30 sep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meracho Senior · Temporada 21 · corte después de la jornada 3 (miércoles 30 sep 2026) · fin de la fase de grupos</t>
+    <t xml:space="preserve">Meracho Senior · Temporada 22 · corte después de la jornada 1 (miércoles 21 oct 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Jugador</t>
   </si>
   <si>
-    <t xml:space="preserve">Angel Rodriguez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luis Aponte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jhon Brenan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oscar Lopez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Erick Zarate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oscar Felibert</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luis Falcon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jair Gonzalez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jair Best</t>
+    <t xml:space="preserve">Roberto Villareal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">José Terriente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">José Delgado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diomedes Frias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tomás Guerra</t>
   </si>
   <si>
     <t xml:space="preserve">Jorge Chevez</t>
   </si>
   <si>
-    <t xml:space="preserve">Virgilio Santos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Josue Vega</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carlos Holder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Micky Sanchez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oscar De Leon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ricardo De Hermoso</t>
+    <t xml:space="preserve">Abi Vargas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kenny Van Gómez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roger Flores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tomás Guerra Jr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adrián Cabezas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juan Carlos Meneses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nicolás Carrega</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mickey Sánchez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tomas Noriega</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sergio González</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Franck Chiary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nedglinyer Marcano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alexis Hartman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abdul Garzón</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Romel Cubilla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eric Yim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Francisco Cárdenas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jack Peter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luis Pineda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Randy Saez</t>
   </si>
   <si>
     <t xml:space="preserve">Roberto Salas</t>
   </si>
   <si>
-    <t xml:space="preserve">Luis Casis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Andy Bravo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Oliver Rubio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jose Acevedo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Edwin Lopez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pablo Duran</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jossue Castillo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Emanuel Diaz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gabriel Caballero</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carlos Merida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Francisco Martin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Javier Nay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Julio Muñoz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roberto Marquez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cristian Bellido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Francisco Mena</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luis Llorente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Martin Paddy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pablo Ortiz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Erick Villarreal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Josue Bragtley</t>
+    <t xml:space="preserve">Gabriel Aira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wilian Aira</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jesus Gil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edgar Hernandez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nicolas Bertrand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wolfang Mendez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reinaldo Arcia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Victor Porras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alexander Salas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angel Lopez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daniel Melendez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Johan Caracas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luis Anzola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mariano Porras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rolando Roquebert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jorge González</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nelson Meléndez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Josue Bragley</t>
+  </si>
+  <si>
+    <t xml:space="preserve">José Camacho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ricardo Martin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">José Luis Frías</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moisés Tenorio</t>
   </si>
   <si>
     <t xml:space="preserve">Abdiel Cerrud</t>
   </si>
   <si>
-    <t xml:space="preserve">José Terriente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alexis Hartman</t>
-  </si>
-  <si>
-    <t xml:space="preserve">William Rodríguez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">José Salas</t>
-  </si>
-  <si>
     <t xml:space="preserve">Daniel Torrealba</t>
   </si>
   <si>
-    <t xml:space="preserve">Abi Vargas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abel Castillo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eric Yim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kenny Van Gómez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">José Luis Frías</t>
+    <t xml:space="preserve">Diego Caballero</t>
   </si>
   <si>
     <t xml:space="preserve">Héctor Vergara</t>
   </si>
   <si>
-    <t xml:space="preserve">Johnatan Santos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">José Camacho</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jorge Batista</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rogelio Chávez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Felix Alveo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jefry Hernandez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jose Lee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Erick Valdivieso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Félix Robles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eduardo Valarezo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alejandro Jaén</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Javier López</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evair Montenegro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juanra Tam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gabriel Riquelme</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jorge León</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jose Medina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juan Carlos Bonilla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jose Gutiérrez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">José Moreno</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ricky Iván Cumberbatch</t>
+    <t xml:space="preserve">Jonathan Santos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Virgilio Parra</t>
   </si>
 </sst>
 </file>
@@ -1200,11 +1146,11 @@
       </c>
       <c r="C5" s="10" t="n">
         <f aca="false">COUNTIF(Resultados!$D$5:$D$200,$B5)+COUNTIF(Resultados!$F$5:$F$200,$B5)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D5" s="10" t="n">
         <f aca="false">SUMPRODUCT((Resultados!$D$5:$D$200=$B5)*(Resultados!$E$5:$E$200&gt;Resultados!$G$5:$G$200))+SUMPRODUCT((Resultados!$F$5:$F$200=$B5)*(Resultados!$G$5:$G$200&gt;Resultados!$E$5:$E$200))</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E5" s="10" t="n">
         <f aca="false">SUMPRODUCT((Resultados!$D$5:$D$200=$B5)*(Resultados!$E$5:$E$200&lt;Resultados!$G$5:$G$200))+SUMPRODUCT((Resultados!$F$5:$F$200=$B5)*(Resultados!$G$5:$G$200&lt;Resultados!$E$5:$E$200))</f>
@@ -1212,15 +1158,15 @@
       </c>
       <c r="F5" s="10" t="n">
         <f aca="false">SUMIF(Resultados!$D$5:$D$200,$B5,Resultados!$E$5:$E$200)+SUMIF(Resultados!$F$5:$F$200,$B5,Resultados!$G$5:$G$200)</f>
-        <v>44</v>
+        <v>15</v>
       </c>
       <c r="G5" s="10" t="n">
         <f aca="false">SUMIF(Resultados!$D$5:$D$200,$B5,Resultados!$G$5:$G$200)+SUMIF(Resultados!$F$5:$F$200,$B5,Resultados!$E$5:$E$200)</f>
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="H5" s="12" t="n">
         <f aca="false">F5-G5</f>
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="I5" s="13" t="n">
         <f aca="false">IF(C5=0,"",D5/C5)</f>
@@ -1236,31 +1182,31 @@
       </c>
       <c r="C6" s="10" t="n">
         <f aca="false">COUNTIF(Resultados!$D$5:$D$200,$B6)+COUNTIF(Resultados!$F$5:$F$200,$B6)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D6" s="10" t="n">
         <f aca="false">SUMPRODUCT((Resultados!$D$5:$D$200=$B6)*(Resultados!$E$5:$E$200&gt;Resultados!$G$5:$G$200))+SUMPRODUCT((Resultados!$F$5:$F$200=$B6)*(Resultados!$G$5:$G$200&gt;Resultados!$E$5:$E$200))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" s="10" t="n">
         <f aca="false">SUMPRODUCT((Resultados!$D$5:$D$200=$B6)*(Resultados!$E$5:$E$200&lt;Resultados!$G$5:$G$200))+SUMPRODUCT((Resultados!$F$5:$F$200=$B6)*(Resultados!$G$5:$G$200&lt;Resultados!$E$5:$E$200))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="10" t="n">
         <f aca="false">SUMIF(Resultados!$D$5:$D$200,$B6,Resultados!$E$5:$E$200)+SUMIF(Resultados!$F$5:$F$200,$B6,Resultados!$G$5:$G$200)</f>
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="G6" s="10" t="n">
         <f aca="false">SUMIF(Resultados!$D$5:$D$200,$B6,Resultados!$G$5:$G$200)+SUMIF(Resultados!$F$5:$F$200,$B6,Resultados!$E$5:$E$200)</f>
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H6" s="12" t="n">
         <f aca="false">F6-G6</f>
-        <v>-3</v>
+        <v>3</v>
       </c>
       <c r="I6" s="13" t="n">
         <f aca="false">IF(C6=0,"",D6/C6)</f>
-        <v>0.666666666666667</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1272,31 +1218,31 @@
       </c>
       <c r="C7" s="10" t="n">
         <f aca="false">COUNTIF(Resultados!$D$5:$D$200,$B7)+COUNTIF(Resultados!$F$5:$F$200,$B7)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D7" s="10" t="n">
         <f aca="false">SUMPRODUCT((Resultados!$D$5:$D$200=$B7)*(Resultados!$E$5:$E$200&gt;Resultados!$G$5:$G$200))+SUMPRODUCT((Resultados!$F$5:$F$200=$B7)*(Resultados!$G$5:$G$200&gt;Resultados!$E$5:$E$200))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" s="10" t="n">
         <f aca="false">SUMPRODUCT((Resultados!$D$5:$D$200=$B7)*(Resultados!$E$5:$E$200&lt;Resultados!$G$5:$G$200))+SUMPRODUCT((Resultados!$F$5:$F$200=$B7)*(Resultados!$G$5:$G$200&lt;Resultados!$E$5:$E$200))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" s="10" t="n">
         <f aca="false">SUMIF(Resultados!$D$5:$D$200,$B7,Resultados!$E$5:$E$200)+SUMIF(Resultados!$F$5:$F$200,$B7,Resultados!$G$5:$G$200)</f>
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="G7" s="10" t="n">
         <f aca="false">SUMIF(Resultados!$D$5:$D$200,$B7,Resultados!$G$5:$G$200)+SUMIF(Resultados!$F$5:$F$200,$B7,Resultados!$E$5:$E$200)</f>
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="H7" s="12" t="n">
         <f aca="false">F7-G7</f>
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="I7" s="13" t="n">
         <f aca="false">IF(C7=0,"",D7/C7)</f>
-        <v>0.333333333333333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1308,7 +1254,7 @@
       </c>
       <c r="C8" s="10" t="n">
         <f aca="false">COUNTIF(Resultados!$D$5:$D$200,$B8)+COUNTIF(Resultados!$F$5:$F$200,$B8)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D8" s="10" t="n">
         <f aca="false">SUMPRODUCT((Resultados!$D$5:$D$200=$B8)*(Resultados!$E$5:$E$200&gt;Resultados!$G$5:$G$200))+SUMPRODUCT((Resultados!$F$5:$F$200=$B8)*(Resultados!$G$5:$G$200&gt;Resultados!$E$5:$E$200))</f>
@@ -1316,19 +1262,19 @@
       </c>
       <c r="E8" s="10" t="n">
         <f aca="false">SUMPRODUCT((Resultados!$D$5:$D$200=$B8)*(Resultados!$E$5:$E$200&lt;Resultados!$G$5:$G$200))+SUMPRODUCT((Resultados!$F$5:$F$200=$B8)*(Resultados!$G$5:$G$200&lt;Resultados!$E$5:$E$200))</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F8" s="10" t="n">
         <f aca="false">SUMIF(Resultados!$D$5:$D$200,$B8,Resultados!$E$5:$E$200)+SUMIF(Resultados!$F$5:$F$200,$B8,Resultados!$G$5:$G$200)</f>
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="G8" s="10" t="n">
         <f aca="false">SUMIF(Resultados!$D$5:$D$200,$B8,Resultados!$G$5:$G$200)+SUMIF(Resultados!$F$5:$F$200,$B8,Resultados!$E$5:$E$200)</f>
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="H8" s="12" t="n">
         <f aca="false">F8-G8</f>
-        <v>-8</v>
+        <v>-5</v>
       </c>
       <c r="I8" s="13" t="n">
         <f aca="false">IF(C8=0,"",D8/C8)</f>
@@ -1420,13 +1366,13 @@
         <v>45</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G5" s="10" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H5" s="10" t="n">
         <v>5</v>
@@ -1443,124 +1389,60 @@
         <v>64</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="E7" s="10" t="n">
-        <v>13</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="G7" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="H7" s="10" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="E8" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="G8" s="10" t="n">
-        <v>11</v>
-      </c>
-      <c r="H8" s="10" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="E9" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="F9" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="G9" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="H9" s="10" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="F10" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="G10" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="H10" s="10" t="n">
-        <v>5</v>
-      </c>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1596,12 +1478,12 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>37</v>
@@ -1645,34 +1527,34 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>45</v>
       </c>
       <c r="C5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="10" t="n">
-        <v>11</v>
-      </c>
       <c r="E5" s="10" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="G5" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" s="10" t="n">
-        <v>9</v>
-      </c>
       <c r="J5" s="13" t="n">
-        <v>0.778</v>
+        <v>1</v>
       </c>
       <c r="K5" s="17"/>
       <c r="L5" s="10"/>
@@ -1681,23 +1563,23 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>45</v>
       </c>
       <c r="C6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="E6" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="F6" s="10" t="n">
-        <v>4</v>
-      </c>
       <c r="G6" s="10" t="n">
         <v>0</v>
       </c>
@@ -1705,10 +1587,10 @@
         <v>0</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J6" s="13" t="n">
-        <v>0.667</v>
+        <v>0.75</v>
       </c>
       <c r="K6" s="17"/>
       <c r="L6" s="10"/>
@@ -1717,34 +1599,34 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>45</v>
       </c>
       <c r="C7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="E7" s="10" t="n">
-        <v>5</v>
-      </c>
       <c r="F7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="10" t="n">
-        <v>5</v>
-      </c>
       <c r="J7" s="13" t="n">
-        <v>0.625</v>
+        <v>0.5</v>
       </c>
       <c r="K7" s="17"/>
       <c r="L7" s="10"/>
@@ -1753,34 +1635,34 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>45</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F8" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="10" t="n">
-        <v>4</v>
-      </c>
       <c r="J8" s="13" t="n">
-        <v>0.875</v>
+        <v>1</v>
       </c>
       <c r="K8" s="17"/>
       <c r="L8" s="10"/>
@@ -1789,34 +1671,34 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>45</v>
       </c>
       <c r="C9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="10" t="n">
-        <v>5</v>
-      </c>
       <c r="E9" s="10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="10" t="n">
-        <v>4</v>
-      </c>
       <c r="J9" s="13" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="K9" s="17"/>
       <c r="L9" s="10"/>
@@ -1825,22 +1707,22 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>45</v>
       </c>
       <c r="C10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="10" t="n">
-        <v>9</v>
-      </c>
       <c r="E10" s="10" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G10" s="10" t="n">
         <v>0</v>
@@ -1849,10 +1731,10 @@
         <v>0</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>0.778</v>
+        <v>1</v>
       </c>
       <c r="K10" s="17"/>
       <c r="L10" s="10"/>
@@ -1861,34 +1743,34 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>45</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J11" s="13" t="n">
-        <v>0.8</v>
+        <v>0.333</v>
       </c>
       <c r="K11" s="17"/>
       <c r="L11" s="10"/>
@@ -1897,34 +1779,34 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>45</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" s="10" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J12" s="13" t="n">
-        <v>0.333</v>
+        <v>1</v>
       </c>
       <c r="K12" s="17"/>
       <c r="L12" s="10"/>
@@ -1933,22 +1815,22 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>45</v>
       </c>
       <c r="C13" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="10" t="n">
-        <v>7</v>
-      </c>
       <c r="E13" s="10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F13" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13" s="10" t="n">
         <v>0</v>
@@ -1960,7 +1842,7 @@
         <v>1</v>
       </c>
       <c r="J13" s="13" t="n">
-        <v>0.429</v>
+        <v>0</v>
       </c>
       <c r="K13" s="17"/>
       <c r="L13" s="10"/>
@@ -1969,22 +1851,22 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>45</v>
       </c>
       <c r="C14" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="10" t="n">
-        <v>5</v>
-      </c>
       <c r="E14" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" s="10" t="n">
         <v>0</v>
@@ -1993,10 +1875,10 @@
         <v>0</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>0.6</v>
+        <v>0.667</v>
       </c>
       <c r="K14" s="17"/>
       <c r="L14" s="10"/>
@@ -2005,19 +1887,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>45</v>
       </c>
       <c r="C15" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D15" s="10" t="n">
-        <v>10</v>
-      </c>
       <c r="E15" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="10" t="n">
         <v>1</v>
@@ -2029,10 +1911,10 @@
         <v>0</v>
       </c>
       <c r="I15" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" s="13" t="n">
-        <v>0.222</v>
+        <v>0.333</v>
       </c>
       <c r="K15" s="17"/>
       <c r="L15" s="10"/>
@@ -2041,7 +1923,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>45</v>
@@ -2050,10 +1932,10 @@
         <v>1</v>
       </c>
       <c r="D16" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" s="10" t="n">
         <v>0</v>
@@ -2065,10 +1947,10 @@
         <v>0</v>
       </c>
       <c r="I16" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16" s="13" t="n">
-        <v>0.333</v>
+        <v>0</v>
       </c>
       <c r="K16" s="17"/>
       <c r="L16" s="10"/>
@@ -2077,7 +1959,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>45</v>
@@ -2113,163 +1995,83 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="13"/>
       <c r="K18" s="17" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L18" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M18" s="10" t="n">
         <v>2</v>
       </c>
       <c r="N18" s="18" t="n">
-        <v>6.3</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C19" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="13"/>
       <c r="K19" s="17"/>
       <c r="L19" s="10"/>
       <c r="M19" s="10"/>
       <c r="N19" s="18"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="13"/>
       <c r="K20" s="17"/>
       <c r="L20" s="10"/>
       <c r="M20" s="10"/>
       <c r="N20" s="18"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C21" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="13" t="n">
-        <v>0</v>
-      </c>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="13"/>
       <c r="K21" s="17"/>
       <c r="L21" s="10"/>
       <c r="M21" s="10"/>
       <c r="N21" s="18"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>45</v>
-      </c>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
@@ -2278,26 +2080,14 @@
       <c r="H22" s="10"/>
       <c r="I22" s="10"/>
       <c r="J22" s="13"/>
-      <c r="K22" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="N22" s="18" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="s">
-        <v>87</v>
-      </c>
-      <c r="B23" s="19" t="s">
-        <v>45</v>
-      </c>
+      <c r="K22" s="17"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="18"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="19"/>
+      <c r="B23" s="19"/>
       <c r="C23" s="20"/>
       <c r="D23" s="20"/>
       <c r="E23" s="20"/>
@@ -2306,18 +2096,10 @@
       <c r="H23" s="20"/>
       <c r="I23" s="20"/>
       <c r="J23" s="20"/>
-      <c r="K23" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="L23" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="M23" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="N23" s="22" t="n">
-        <v>1.75</v>
-      </c>
+      <c r="K23" s="21"/>
+      <c r="L23" s="20"/>
+      <c r="M23" s="20"/>
+      <c r="N23" s="22"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2353,12 +2135,12 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>37</v>
@@ -2402,34 +2184,34 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="10" t="n">
-        <v>8</v>
-      </c>
       <c r="E5" s="10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="G5" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="10" t="n">
-        <v>5</v>
-      </c>
       <c r="J5" s="13" t="n">
-        <v>0.714</v>
+        <v>0.667</v>
       </c>
       <c r="K5" s="17"/>
       <c r="L5" s="10"/>
@@ -2438,19 +2220,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="E6" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>0</v>
@@ -2459,13 +2241,13 @@
         <v>0</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>3</v>
       </c>
       <c r="J6" s="13" t="n">
-        <v>0.333</v>
+        <v>0.5</v>
       </c>
       <c r="K6" s="17"/>
       <c r="L6" s="10"/>
@@ -2474,19 +2256,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="10" t="n">
-        <v>8</v>
-      </c>
       <c r="E7" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>0</v>
@@ -2501,7 +2283,7 @@
         <v>2</v>
       </c>
       <c r="J7" s="13" t="n">
-        <v>0.429</v>
+        <v>0.333</v>
       </c>
       <c r="K7" s="17"/>
       <c r="L7" s="10"/>
@@ -2510,22 +2292,22 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" s="10" t="n">
         <v>0</v>
@@ -2537,7 +2319,7 @@
         <v>2</v>
       </c>
       <c r="J8" s="13" t="n">
-        <v>0.333</v>
+        <v>0.5</v>
       </c>
       <c r="K8" s="17"/>
       <c r="L8" s="10"/>
@@ -2546,16 +2328,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="10" t="n">
         <v>3</v>
-      </c>
-      <c r="D9" s="10" t="n">
-        <v>9</v>
       </c>
       <c r="E9" s="10" t="n">
         <v>3</v>
@@ -2573,7 +2355,7 @@
         <v>1</v>
       </c>
       <c r="J9" s="13" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="K9" s="17"/>
       <c r="L9" s="10"/>
@@ -2582,19 +2364,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="E10" s="10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F10" s="10" t="n">
         <v>0</v>
@@ -2609,7 +2391,7 @@
         <v>1</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="K10" s="17"/>
       <c r="L10" s="10"/>
@@ -2618,22 +2400,22 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="10" t="n">
         <v>0</v>
@@ -2642,10 +2424,10 @@
         <v>0</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11" s="13" t="n">
-        <v>0.286</v>
+        <v>1</v>
       </c>
       <c r="K11" s="17"/>
       <c r="L11" s="10"/>
@@ -2654,22 +2436,22 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12" s="10" t="n">
         <v>0</v>
@@ -2678,11 +2460,9 @@
         <v>0</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="13" t="n">
-        <v>0.333</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J12" s="13"/>
       <c r="K12" s="17"/>
       <c r="L12" s="10"/>
       <c r="M12" s="10"/>
@@ -2690,7 +2470,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>47</v>
@@ -2699,10 +2479,10 @@
         <v>1</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" s="10" t="n">
         <v>0</v>
@@ -2714,10 +2494,10 @@
         <v>0</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" s="17"/>
       <c r="L13" s="10"/>
@@ -2726,19 +2506,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" s="10" t="n">
         <v>0</v>
@@ -2750,10 +2530,10 @@
         <v>0</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>0.333</v>
+        <v>0</v>
       </c>
       <c r="K14" s="17"/>
       <c r="L14" s="10"/>
@@ -2762,19 +2542,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D15" s="10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" s="10" t="n">
         <v>0</v>
@@ -2786,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="I15" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" s="13" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="K15" s="17"/>
       <c r="L15" s="10"/>
@@ -2798,55 +2578,63 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C16" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D16" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="L16" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="13" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="K16" s="17"/>
-      <c r="L16" s="10"/>
-      <c r="M16" s="10"/>
-      <c r="N16" s="18"/>
+      <c r="N16" s="18" t="n">
+        <v>12.25</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>47</v>
       </c>
       <c r="C17" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" s="10" t="n">
         <v>0</v>
@@ -2861,7 +2649,7 @@
         <v>0</v>
       </c>
       <c r="J17" s="13" t="n">
-        <v>0.333</v>
+        <v>0</v>
       </c>
       <c r="K17" s="17"/>
       <c r="L17" s="10"/>
@@ -2869,105 +2657,47 @@
       <c r="N17" s="18"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C18" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D18" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="E18" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="13" t="n">
-        <v>0.2</v>
-      </c>
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="13"/>
       <c r="K18" s="17"/>
       <c r="L18" s="10"/>
       <c r="M18" s="10"/>
       <c r="N18" s="18"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D19" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E19" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="13" t="n">
-        <v>0.333</v>
-      </c>
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="13"/>
       <c r="K19" s="17"/>
       <c r="L19" s="10"/>
       <c r="M19" s="10"/>
       <c r="N19" s="18"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C20" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="10" t="n">
-        <v>0</v>
-      </c>
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
       <c r="J20" s="13"/>
       <c r="K20" s="17"/>
       <c r="L20" s="10"/>
@@ -2975,48 +2705,24 @@
       <c r="N20" s="18"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C21" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="13"/>
       <c r="K21" s="17"/>
       <c r="L21" s="10"/>
       <c r="M21" s="10"/>
       <c r="N21" s="18"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>47</v>
-      </c>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
@@ -3025,26 +2731,14 @@
       <c r="H22" s="10"/>
       <c r="I22" s="10"/>
       <c r="J22" s="13"/>
-      <c r="K22" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="L22" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="18" t="n">
-        <v>5.25</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>47</v>
-      </c>
+      <c r="K22" s="17"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="18"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
@@ -3053,20 +2747,12 @@
       <c r="H23" s="10"/>
       <c r="I23" s="10"/>
       <c r="J23" s="13"/>
-      <c r="K23" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="L23" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="M23" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="N23" s="18" t="n">
-        <v>9.92</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K23" s="17"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="18"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="23"/>
       <c r="B24" s="24"/>
       <c r="C24" s="24"/>
@@ -3094,6 +2780,681 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:N22"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="3" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="M4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="N4" s="16" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K5" s="17"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="18"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="17"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="18"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="13" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="K7" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="L7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" s="18" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="13" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="K8" s="17"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="18"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="17"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="18"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="17"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="18"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="17"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="18"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="17"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10"/>
+      <c r="N12" s="18"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="17"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="18"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="13"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="18"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="17"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="18"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="17"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10"/>
+      <c r="N16" s="18"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="17"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="18"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="17"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="18"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="17"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="18"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="17"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="18"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="17"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="18"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="19"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="20"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="21"/>
+      <c r="L22" s="20"/>
+      <c r="M22" s="20"/>
+      <c r="N22" s="22"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -3116,12 +3477,12 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>37</v>
@@ -3165,76 +3526,70 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="10" t="n">
-        <v>8</v>
-      </c>
       <c r="E5" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J5" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K5" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="10" t="n">
-        <v>0</v>
-      </c>
+        <v>0.333</v>
+      </c>
+      <c r="K5" s="17"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
       <c r="N5" s="18"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="10" t="n">
-        <v>9</v>
-      </c>
       <c r="E6" s="10" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G6" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="10" t="n">
-        <v>4</v>
-      </c>
       <c r="J6" s="13" t="n">
-        <v>0.75</v>
+        <v>0.667</v>
       </c>
       <c r="K6" s="17"/>
       <c r="L6" s="10"/>
@@ -3243,76 +3598,78 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D7" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="17" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="L7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="E7" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="F7" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="J7" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K7" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="18"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H8" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J8" s="13" t="n">
-        <v>0.429</v>
+        <v>0.5</v>
       </c>
       <c r="K8" s="17"/>
       <c r="L8" s="10"/>
@@ -3321,19 +3678,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>0</v>
@@ -3345,10 +3702,10 @@
         <v>0</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" s="13" t="n">
-        <v>0.833</v>
+        <v>1</v>
       </c>
       <c r="K9" s="17"/>
       <c r="L9" s="10"/>
@@ -3357,22 +3714,22 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C10" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G10" s="10" t="n">
         <v>0</v>
@@ -3381,10 +3738,10 @@
         <v>0</v>
       </c>
       <c r="I10" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="K10" s="17"/>
       <c r="L10" s="10"/>
@@ -3393,16 +3750,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C11" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E11" s="10" t="n">
         <v>2</v>
@@ -3411,33 +3768,25 @@
         <v>0</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H11" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J11" s="13" t="n">
-        <v>0.286</v>
-      </c>
-      <c r="K11" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="L11" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="18" t="n">
-        <v>18.67</v>
-      </c>
+        <v>0.667</v>
+      </c>
+      <c r="K11" s="17"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>51</v>
@@ -3461,7 +3810,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J12" s="13" t="n">
         <v>0.333</v>
@@ -3473,69 +3822,61 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C13" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D13" s="10" t="n">
-        <v>7</v>
-      </c>
       <c r="E13" s="10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F13" s="10" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" s="10" t="n">
         <v>0</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13" s="13" t="n">
-        <v>0.667</v>
-      </c>
-      <c r="K13" s="17" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="L13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="N13" s="18" t="n">
-        <v>10.5</v>
-      </c>
+        <v>0.333</v>
+      </c>
+      <c r="K13" s="17"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14" s="10" t="n">
         <v>0</v>
@@ -3544,7 +3885,7 @@
         <v>0</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K14" s="17"/>
       <c r="L14" s="10"/>
@@ -3553,25 +3894,25 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C15" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="10" t="n">
-        <v>6</v>
-      </c>
       <c r="E15" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="10" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15" s="10" t="n">
         <v>0</v>
@@ -3580,7 +3921,7 @@
         <v>0</v>
       </c>
       <c r="J15" s="13" t="n">
-        <v>0.333</v>
+        <v>0.5</v>
       </c>
       <c r="K15" s="17"/>
       <c r="L15" s="10"/>
@@ -3589,7 +3930,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>51</v>
@@ -3598,7 +3939,7 @@
         <v>1</v>
       </c>
       <c r="D16" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E16" s="10" t="n">
         <v>1</v>
@@ -3616,7 +3957,7 @@
         <v>0</v>
       </c>
       <c r="J16" s="13" t="n">
-        <v>0.5</v>
+        <v>0.333</v>
       </c>
       <c r="K16" s="17"/>
       <c r="L16" s="10"/>
@@ -3625,16 +3966,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C17" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E17" s="10" t="n">
         <v>0</v>
@@ -3654,54 +3995,38 @@
       <c r="J17" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="K17" s="17"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="10"/>
-      <c r="N17" s="18"/>
+      <c r="K17" s="17" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="L17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="18" t="n">
+        <v>31.5</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C18" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="A18" s="5"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="13"/>
       <c r="K18" s="17"/>
       <c r="L18" s="10"/>
       <c r="M18" s="10"/>
       <c r="N18" s="18"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>51</v>
-      </c>
+      <c r="A19" s="5"/>
+      <c r="B19" s="5"/>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
@@ -3710,20 +4035,12 @@
       <c r="H19" s="10"/>
       <c r="I19" s="10"/>
       <c r="J19" s="13"/>
-      <c r="K19" s="17" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="L19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="18" t="n">
-        <v>11.87</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K19" s="17"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="18"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="23"/>
       <c r="B20" s="24"/>
       <c r="C20" s="24"/>
@@ -3748,733 +4065,4 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:N22"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="3" style="1" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="1" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="8"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="K4" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="L4" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="M4" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="N4" s="16" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C5" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D5" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="E5" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="F5" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="G5" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="J5" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" s="17"/>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="18"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E6" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="F6" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="G6" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="J6" s="13" t="n">
-        <v>0.667</v>
-      </c>
-      <c r="K6" s="17" t="n">
-        <v>15</v>
-      </c>
-      <c r="L6" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M6" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="N6" s="18" t="n">
-        <v>9.8</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="E7" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="F7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="J7" s="13" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="K7" s="17"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="18"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="E8" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="J8" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K8" s="17"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="18"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D9" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="E9" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="F9" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="J9" s="13" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="K9" s="17"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="18"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="E10" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="F10" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="J10" s="13" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="K10" s="17"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
-      <c r="N10" s="18"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="E11" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="J11" s="13" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="K11" s="17"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="10"/>
-      <c r="N11" s="18"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D12" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="E12" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="F12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="13" t="n">
-        <v>0.714</v>
-      </c>
-      <c r="K12" s="17"/>
-      <c r="L12" s="10"/>
-      <c r="M12" s="10"/>
-      <c r="N12" s="18"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="E13" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="F13" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="G13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J13" s="13" t="n">
-        <v>0.714</v>
-      </c>
-      <c r="K13" s="17"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="18"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D14" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="E14" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="F14" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="G14" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J14" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K14" s="17"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="18"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D15" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="E15" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="F15" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="K15" s="17"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="18"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C16" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E16" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" s="13" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="K16" s="17"/>
-      <c r="L16" s="10"/>
-      <c r="M16" s="10"/>
-      <c r="N16" s="18"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C17" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E17" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K17" s="17"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="10"/>
-      <c r="N17" s="18"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C18" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="E18" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="F18" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K18" s="17"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="10"/>
-      <c r="N18" s="18"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C19" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="D19" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="E19" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="13" t="n">
-        <v>0.222</v>
-      </c>
-      <c r="K19" s="17"/>
-      <c r="L19" s="10"/>
-      <c r="M19" s="10"/>
-      <c r="N19" s="18"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C20" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" s="17"/>
-      <c r="L20" s="10"/>
-      <c r="M20" s="10"/>
-      <c r="N20" s="18"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="C21" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="17"/>
-      <c r="L21" s="10"/>
-      <c r="M21" s="10"/>
-      <c r="N21" s="18"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="s">
-        <v>139</v>
-      </c>
-      <c r="B22" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="20"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="20"/>
-      <c r="H22" s="20"/>
-      <c r="I22" s="20"/>
-      <c r="J22" s="20"/>
-      <c r="K22" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="22" t="n">
-        <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>